<commit_message>
Căn cấu hình theo file thực tế và sửa lỗi khớp mặt hàng
- MAIN: tiêu đề dòng 9-10, dữ liệu từ dòng 11; cột theo vị trí thật
  (MST=9, Số HĐ=5, Ngày=7, Giá trị chưa thuế=14, Thuế GTGT=17, Hàng=10).
- RISK: hỗ trợ nhiều sheet khác cấu trúc, gộp MST + văn bản từ cả 3 sheet;
  doc_col nhận số (cột theo dòng) hoặc chữ (nhãn văn bản cố định).
- Sửa lỗi tác vụ 7: giữ nguyên dấu tiếng Việt khi dò từ khóa, tránh nhầm
  "tặng" với "tầng/tăng" (giảm cảnh báo sai từ ~1000 xuống còn đúng thực tế).
- Bỏ qua file HĐĐT rỗng (tránh gắn nhầm nhãn "không tìm thấy" toàn bộ).
- utils: đọc được sheet theo tên, tua lại con trỏ file upload để đọc nhiều lần.
- Cập nhật app (cấu hình DS rủi ro nhiều sheet, cảnh báo HĐĐT rỗng),
  make_samples và README theo bố cục thật.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Axb5Z5tNQVDeR5iir9sJuR
</commit_message>
<xml_diff>
--- a/samples/01_du_lieu_chinh.xlsx
+++ b/samples/01_du_lieu_chinh.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BK MV- 2020-2025 (đã sửa)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,235 +413,439 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="B1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>MST</t>
-        </is>
-      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Số hóa đơn</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Ngày hóa đơn</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Giá trị chưa thuế</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Thuế GTGT</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Tên hàng hóa</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>0101234567</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+          <t>BẢNG KÊ HOÁ ĐƠN, CHỨNG TỪ HÀNG HOÁ, DỊCH VỤ MUA VÀO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CÔNG TY MẪU DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0304436870</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tên người bán</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Mã số thuế người bán</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Tên hàng hóa, dịch vụ</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Giá trị HHDV mua vào chưa có thuế GTGT</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Tiền thuế GTGT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mẫu số</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ký hiệu</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Số</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Ngày, tháng, năm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AA/20E</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>0000123</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2020-10-23</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Ngân hàng ABC</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0301224067</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Phí ngân hàng</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>525000</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>AA/20E</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0000123</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2020-10-23</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Ngân hàng ABC</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0301224067</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Phí ngân hàng</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>525000</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ME/20E</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0000045</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2021-02-20</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Công ty Rượu XYZ</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0312816241</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Chai rượu vang biếu khách</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ME/20E</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0000046</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2021-03-01</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Công ty Golf</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0313025323</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Bộ gậy chơi golf</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HK/18P</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0000789</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2022-04-10</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Công ty Vật tư</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0400111222</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Thép hộp tăng cường (không trùng golf)</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>HK/18P</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0000790</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>790</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2022-06-15</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Công ty Quà</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0400111222</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Quà tặng khách hàng</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CA/19P</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2023-05-05</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Công ty VPP</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Văn phòng phẩm</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
         <v>1000000</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Dịch vụ tư vấn</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>0101234567</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Dịch vụ tư vấn (trùng)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>0312345678</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>0045</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="E4" t="n">
-        <v>500000</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Chai rượu vang biếu khách</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>0312345678</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0046</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="E5" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Bộ gậy chơi golf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>0400111222</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>0789</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>800000</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Vật tư sản xuất</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>0400111222</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>0790</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Quà tặng khách hàng</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>9999999999</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="Q17" t="n">
         <v>100000</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Văn phòng phẩm</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>